<commit_message>
updated all tables for r8
</commit_message>
<xml_diff>
--- a/htan2-data-release-pipeline/medallion_architecture/gold2isbcgc/log/Metadata_Table_Descriptions_R8.xlsx
+++ b/htan2-data-release-pipeline/medallion_architecture/gold2isbcgc/log/Metadata_Table_Descriptions_R8.xlsx
@@ -582,10 +582,10 @@
         </is>
       </c>
       <c r="O2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="P2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">
@@ -660,10 +660,10 @@
         </is>
       </c>
       <c r="O3" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="P3" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4">
@@ -738,10 +738,10 @@
         </is>
       </c>
       <c r="O4" t="n">
-        <v>39</v>
+        <v>24</v>
       </c>
       <c r="P4" t="n">
-        <v>39</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5">
@@ -816,10 +816,10 @@
         </is>
       </c>
       <c r="O5" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="P5" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
@@ -894,10 +894,10 @@
         </is>
       </c>
       <c r="O6" t="n">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="P6" t="n">
-        <v>29</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7">
@@ -972,10 +972,10 @@
         </is>
       </c>
       <c r="O7" t="n">
-        <v>71</v>
+        <v>53</v>
       </c>
       <c r="P7" t="n">
-        <v>71</v>
+        <v>53</v>
       </c>
     </row>
     <row r="8">
@@ -1050,10 +1050,10 @@
         </is>
       </c>
       <c r="O8" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="P8" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9">
@@ -1128,10 +1128,10 @@
         </is>
       </c>
       <c r="O9" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="P9" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="10">
@@ -1206,10 +1206,10 @@
         </is>
       </c>
       <c r="O10" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="P10" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11">
@@ -1284,10 +1284,10 @@
         </is>
       </c>
       <c r="O11" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="P11" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12">
@@ -1362,10 +1362,10 @@
         </is>
       </c>
       <c r="O12" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="P12" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13">
@@ -1440,10 +1440,10 @@
         </is>
       </c>
       <c r="O13" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="P13" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14">
@@ -1596,10 +1596,10 @@
         </is>
       </c>
       <c r="O15" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="P15" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="16">
@@ -1674,10 +1674,10 @@
         </is>
       </c>
       <c r="O16" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="P16" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="17">
@@ -1830,10 +1830,10 @@
         </is>
       </c>
       <c r="O18" t="n">
-        <v>99</v>
+        <v>65</v>
       </c>
       <c r="P18" t="n">
-        <v>99</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>